<commit_message>
chore: commit current gxp audit baseline
</commit_message>
<xml_diff>
--- a/docs/csv-validation/IntRuoyi-eDHR-CSV现场证据包.xlsx
+++ b/docs/csv-validation/IntRuoyi-eDHR-CSV现场证据包.xlsx
@@ -3,20 +3,20 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面说明" sheetId="1" r:id="rId1"/>
-    <x:sheet name="7.1培训矩阵" sheetId="2" r:id="R287161a9f5b54086"/>
-    <x:sheet name="7.1培训记录" sheetId="3" r:id="R64f8cb6203e44549"/>
-    <x:sheet name="7.2手册清单" sheetId="4" r:id="Rf40bfb4235ee435a"/>
-    <x:sheet name="7.3文档主清单" sheetId="5" r:id="R4b5e45bc6f7447d7"/>
-    <x:sheet name="7.4岗位匹配" sheetId="6" r:id="R1559b132ecad465e"/>
-    <x:sheet name="权限培训关联" sheetId="7" r:id="Ra45674dae7834f38"/>
-    <x:sheet name="CAPA整改跟踪" sheetId="8" r:id="Re03f6271cbe14ace"/>
-    <x:sheet name="抽查检查表" sheetId="9" r:id="Rcf5333926131495f"/>
-    <x:sheet name="系统依据" sheetId="10" r:id="Rf058d2d71d434e06"/>
-    <x:sheet name="签字与批准矩阵" sheetId="11" r:id="R1a8463ddbd0f4661"/>
-    <x:sheet name="现场填报索引" sheetId="12" r:id="Rf6acc1ae9bb34143"/>
-    <x:sheet name="文件发放回收" sheetId="13" r:id="R9c18fcd122dd4839"/>
-    <x:sheet name="培训人员记录" sheetId="14" r:id="R13da7d39bbd24131"/>
-    <x:sheet name="证据附件索引" sheetId="15" r:id="R511a893bac1d493f"/>
+    <x:sheet name="7.1培训矩阵" sheetId="2" r:id="R8a8530f65ae441c9"/>
+    <x:sheet name="7.1培训记录" sheetId="3" r:id="Raf3b944a219a41b0"/>
+    <x:sheet name="7.2手册清单" sheetId="4" r:id="R9592cff0e3ef4732"/>
+    <x:sheet name="7.3文档主清单" sheetId="5" r:id="R1dc480f7b68e4aa6"/>
+    <x:sheet name="7.4岗位匹配" sheetId="6" r:id="R5a94378fb1da4824"/>
+    <x:sheet name="权限培训关联" sheetId="7" r:id="Rf5ade0f4e52c4038"/>
+    <x:sheet name="CAPA整改跟踪" sheetId="8" r:id="Rb6d4468010134bc2"/>
+    <x:sheet name="抽查检查表" sheetId="9" r:id="R321ac880e3bc4ad9"/>
+    <x:sheet name="系统依据" sheetId="10" r:id="Re6017d46800a41f0"/>
+    <x:sheet name="签字与批准矩阵" sheetId="11" r:id="Re3e3483f00b344ee"/>
+    <x:sheet name="现场填报索引" sheetId="12" r:id="R750c30a853ac436c"/>
+    <x:sheet name="文件发放回收" sheetId="13" r:id="R3c7841523a5f4cbd"/>
+    <x:sheet name="培训人员记录" sheetId="14" r:id="Rc415889d53fd45e2"/>
+    <x:sheet name="证据附件索引" sheetId="15" r:id="R667bb0427d1c4e21"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">封面说明!A1:C11</x:definedName>

</xml_diff>